<commit_message>
Reset Excel Table for CUTTING-01
</commit_message>
<xml_diff>
--- a/FM-MN-07_CUTTING-01.xlsx
+++ b/FM-MN-07_CUTTING-01.xlsx
@@ -1726,41 +1726,37 @@
           <t xml:space="preserve">การ Worm spindle ก่อนเริ่มงาน เพื่อตรวจ ความผิดปกติของชุด Back gauge และ Motor </t>
         </is>
       </c>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="20" t="n"/>
-      <c r="F6" s="20" t="n"/>
-      <c r="G6" s="20" t="n"/>
-      <c r="H6" s="20" t="n"/>
-      <c r="I6" s="20" t="n"/>
-      <c r="J6" s="20" t="n"/>
-      <c r="K6" s="20" t="n"/>
-      <c r="L6" s="20" t="n"/>
-      <c r="M6" s="20" t="n"/>
-      <c r="N6" s="20" t="n"/>
-      <c r="O6" s="20" t="n"/>
-      <c r="P6" s="20" t="n"/>
-      <c r="Q6" s="20" t="n"/>
-      <c r="R6" s="20" t="n"/>
-      <c r="S6" s="20" t="n"/>
-      <c r="T6" s="20" t="n"/>
-      <c r="U6" s="20" t="n"/>
-      <c r="V6" s="20" t="n"/>
-      <c r="W6" s="20" t="n"/>
-      <c r="X6" s="20" t="n"/>
-      <c r="Y6" s="20" t="n"/>
-      <c r="Z6" s="20" t="n"/>
-      <c r="AA6" s="20" t="n"/>
-      <c r="AB6" s="20" t="n"/>
-      <c r="AC6" s="20" t="n"/>
-      <c r="AD6" s="20" t="n"/>
-      <c r="AE6" s="20" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AF6" s="20" t="n"/>
-      <c r="AG6" s="20" t="n"/>
+      <c r="C6" s="20" t="inlineStr"/>
+      <c r="D6" s="20" t="inlineStr"/>
+      <c r="E6" s="20" t="inlineStr"/>
+      <c r="F6" s="20" t="inlineStr"/>
+      <c r="G6" s="20" t="inlineStr"/>
+      <c r="H6" s="20" t="inlineStr"/>
+      <c r="I6" s="20" t="inlineStr"/>
+      <c r="J6" s="20" t="inlineStr"/>
+      <c r="K6" s="20" t="inlineStr"/>
+      <c r="L6" s="20" t="inlineStr"/>
+      <c r="M6" s="20" t="inlineStr"/>
+      <c r="N6" s="20" t="inlineStr"/>
+      <c r="O6" s="20" t="inlineStr"/>
+      <c r="P6" s="20" t="inlineStr"/>
+      <c r="Q6" s="20" t="inlineStr"/>
+      <c r="R6" s="20" t="inlineStr"/>
+      <c r="S6" s="20" t="inlineStr"/>
+      <c r="T6" s="20" t="inlineStr"/>
+      <c r="U6" s="20" t="inlineStr"/>
+      <c r="V6" s="20" t="inlineStr"/>
+      <c r="W6" s="20" t="inlineStr"/>
+      <c r="X6" s="20" t="inlineStr"/>
+      <c r="Y6" s="20" t="inlineStr"/>
+      <c r="Z6" s="20" t="inlineStr"/>
+      <c r="AA6" s="20" t="inlineStr"/>
+      <c r="AB6" s="20" t="inlineStr"/>
+      <c r="AC6" s="20" t="inlineStr"/>
+      <c r="AD6" s="20" t="inlineStr"/>
+      <c r="AE6" s="20" t="inlineStr"/>
+      <c r="AF6" s="20" t="inlineStr"/>
+      <c r="AG6" s="20" t="inlineStr"/>
     </row>
     <row r="7" ht="15.75" customFormat="1" customHeight="1" s="10">
       <c r="A7" s="9" t="n">
@@ -1771,41 +1767,37 @@
           <t>เช็ค Auto Up-Down back gauge และ Manual ( ความคล่องตัวในการเคลื่อนที่ )</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n"/>
-      <c r="D7" s="20" t="n"/>
-      <c r="E7" s="20" t="n"/>
-      <c r="F7" s="20" t="n"/>
-      <c r="G7" s="20" t="n"/>
-      <c r="H7" s="20" t="n"/>
-      <c r="I7" s="20" t="n"/>
-      <c r="J7" s="20" t="n"/>
-      <c r="K7" s="20" t="n"/>
-      <c r="L7" s="20" t="n"/>
-      <c r="M7" s="20" t="n"/>
-      <c r="N7" s="20" t="n"/>
-      <c r="O7" s="20" t="n"/>
-      <c r="P7" s="20" t="n"/>
-      <c r="Q7" s="20" t="n"/>
-      <c r="R7" s="20" t="n"/>
-      <c r="S7" s="20" t="n"/>
-      <c r="T7" s="20" t="n"/>
-      <c r="U7" s="20" t="n"/>
-      <c r="V7" s="20" t="n"/>
-      <c r="W7" s="20" t="n"/>
-      <c r="X7" s="20" t="n"/>
-      <c r="Y7" s="20" t="n"/>
-      <c r="Z7" s="20" t="n"/>
-      <c r="AA7" s="20" t="n"/>
-      <c r="AB7" s="20" t="n"/>
-      <c r="AC7" s="20" t="n"/>
-      <c r="AD7" s="20" t="n"/>
-      <c r="AE7" s="20" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="AF7" s="20" t="n"/>
-      <c r="AG7" s="20" t="n"/>
+      <c r="C7" s="20" t="inlineStr"/>
+      <c r="D7" s="20" t="inlineStr"/>
+      <c r="E7" s="20" t="inlineStr"/>
+      <c r="F7" s="20" t="inlineStr"/>
+      <c r="G7" s="20" t="inlineStr"/>
+      <c r="H7" s="20" t="inlineStr"/>
+      <c r="I7" s="20" t="inlineStr"/>
+      <c r="J7" s="20" t="inlineStr"/>
+      <c r="K7" s="20" t="inlineStr"/>
+      <c r="L7" s="20" t="inlineStr"/>
+      <c r="M7" s="20" t="inlineStr"/>
+      <c r="N7" s="20" t="inlineStr"/>
+      <c r="O7" s="20" t="inlineStr"/>
+      <c r="P7" s="20" t="inlineStr"/>
+      <c r="Q7" s="20" t="inlineStr"/>
+      <c r="R7" s="20" t="inlineStr"/>
+      <c r="S7" s="20" t="inlineStr"/>
+      <c r="T7" s="20" t="inlineStr"/>
+      <c r="U7" s="20" t="inlineStr"/>
+      <c r="V7" s="20" t="inlineStr"/>
+      <c r="W7" s="20" t="inlineStr"/>
+      <c r="X7" s="20" t="inlineStr"/>
+      <c r="Y7" s="20" t="inlineStr"/>
+      <c r="Z7" s="20" t="inlineStr"/>
+      <c r="AA7" s="20" t="inlineStr"/>
+      <c r="AB7" s="20" t="inlineStr"/>
+      <c r="AC7" s="20" t="inlineStr"/>
+      <c r="AD7" s="20" t="inlineStr"/>
+      <c r="AE7" s="20" t="inlineStr"/>
+      <c r="AF7" s="20" t="inlineStr"/>
+      <c r="AG7" s="20" t="inlineStr"/>
     </row>
     <row r="8" ht="15.75" customFormat="1" customHeight="1" s="10">
       <c r="A8" s="9" t="n">
@@ -1816,41 +1808,37 @@
           <t>ระดับน้ำมันไฮดรอลิค ตรวจสอบระดับในปั้มน้ำมัน หล่อลืนแกน  Back gauge</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n"/>
-      <c r="D8" s="20" t="n"/>
-      <c r="E8" s="20" t="n"/>
-      <c r="F8" s="20" t="n"/>
-      <c r="G8" s="20" t="n"/>
-      <c r="H8" s="20" t="n"/>
-      <c r="I8" s="20" t="n"/>
-      <c r="J8" s="20" t="n"/>
-      <c r="K8" s="20" t="n"/>
-      <c r="L8" s="20" t="n"/>
-      <c r="M8" s="20" t="n"/>
-      <c r="N8" s="20" t="n"/>
-      <c r="O8" s="20" t="n"/>
-      <c r="P8" s="20" t="n"/>
-      <c r="Q8" s="20" t="n"/>
-      <c r="R8" s="20" t="n"/>
-      <c r="S8" s="20" t="n"/>
-      <c r="T8" s="20" t="n"/>
-      <c r="U8" s="20" t="n"/>
-      <c r="V8" s="20" t="n"/>
-      <c r="W8" s="20" t="n"/>
-      <c r="X8" s="20" t="n"/>
-      <c r="Y8" s="20" t="n"/>
-      <c r="Z8" s="20" t="n"/>
-      <c r="AA8" s="20" t="n"/>
-      <c r="AB8" s="20" t="n"/>
-      <c r="AC8" s="20" t="n"/>
-      <c r="AD8" s="20" t="n"/>
-      <c r="AE8" s="20" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF8" s="20" t="n"/>
-      <c r="AG8" s="20" t="n"/>
+      <c r="C8" s="20" t="inlineStr"/>
+      <c r="D8" s="20" t="inlineStr"/>
+      <c r="E8" s="20" t="inlineStr"/>
+      <c r="F8" s="20" t="inlineStr"/>
+      <c r="G8" s="20" t="inlineStr"/>
+      <c r="H8" s="20" t="inlineStr"/>
+      <c r="I8" s="20" t="inlineStr"/>
+      <c r="J8" s="20" t="inlineStr"/>
+      <c r="K8" s="20" t="inlineStr"/>
+      <c r="L8" s="20" t="inlineStr"/>
+      <c r="M8" s="20" t="inlineStr"/>
+      <c r="N8" s="20" t="inlineStr"/>
+      <c r="O8" s="20" t="inlineStr"/>
+      <c r="P8" s="20" t="inlineStr"/>
+      <c r="Q8" s="20" t="inlineStr"/>
+      <c r="R8" s="20" t="inlineStr"/>
+      <c r="S8" s="20" t="inlineStr"/>
+      <c r="T8" s="20" t="inlineStr"/>
+      <c r="U8" s="20" t="inlineStr"/>
+      <c r="V8" s="20" t="inlineStr"/>
+      <c r="W8" s="20" t="inlineStr"/>
+      <c r="X8" s="20" t="inlineStr"/>
+      <c r="Y8" s="20" t="inlineStr"/>
+      <c r="Z8" s="20" t="inlineStr"/>
+      <c r="AA8" s="20" t="inlineStr"/>
+      <c r="AB8" s="20" t="inlineStr"/>
+      <c r="AC8" s="20" t="inlineStr"/>
+      <c r="AD8" s="20" t="inlineStr"/>
+      <c r="AE8" s="20" t="inlineStr"/>
+      <c r="AF8" s="20" t="inlineStr"/>
+      <c r="AG8" s="20" t="inlineStr"/>
     </row>
     <row r="9" ht="15.75" customFormat="1" customHeight="1" s="10">
       <c r="A9" s="9" t="n">
@@ -1861,41 +1849,37 @@
           <t>ตรวจเช็ค  Switch  เปิด-ปิด</t>
         </is>
       </c>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="n"/>
-      <c r="F9" s="20" t="n"/>
-      <c r="G9" s="20" t="n"/>
-      <c r="H9" s="20" t="n"/>
-      <c r="I9" s="20" t="n"/>
-      <c r="J9" s="20" t="n"/>
-      <c r="K9" s="20" t="n"/>
-      <c r="L9" s="20" t="n"/>
-      <c r="M9" s="20" t="n"/>
-      <c r="N9" s="20" t="n"/>
-      <c r="O9" s="20" t="n"/>
-      <c r="P9" s="20" t="n"/>
-      <c r="Q9" s="20" t="n"/>
-      <c r="R9" s="20" t="n"/>
-      <c r="S9" s="20" t="n"/>
-      <c r="T9" s="20" t="n"/>
-      <c r="U9" s="20" t="n"/>
-      <c r="V9" s="20" t="n"/>
-      <c r="W9" s="20" t="n"/>
-      <c r="X9" s="20" t="n"/>
-      <c r="Y9" s="20" t="n"/>
-      <c r="Z9" s="20" t="n"/>
-      <c r="AA9" s="20" t="n"/>
-      <c r="AB9" s="20" t="n"/>
-      <c r="AC9" s="20" t="n"/>
-      <c r="AD9" s="20" t="n"/>
-      <c r="AE9" s="20" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF9" s="20" t="n"/>
-      <c r="AG9" s="20" t="n"/>
+      <c r="C9" s="20" t="inlineStr"/>
+      <c r="D9" s="20" t="inlineStr"/>
+      <c r="E9" s="20" t="inlineStr"/>
+      <c r="F9" s="20" t="inlineStr"/>
+      <c r="G9" s="20" t="inlineStr"/>
+      <c r="H9" s="20" t="inlineStr"/>
+      <c r="I9" s="20" t="inlineStr"/>
+      <c r="J9" s="20" t="inlineStr"/>
+      <c r="K9" s="20" t="inlineStr"/>
+      <c r="L9" s="20" t="inlineStr"/>
+      <c r="M9" s="20" t="inlineStr"/>
+      <c r="N9" s="20" t="inlineStr"/>
+      <c r="O9" s="20" t="inlineStr"/>
+      <c r="P9" s="20" t="inlineStr"/>
+      <c r="Q9" s="20" t="inlineStr"/>
+      <c r="R9" s="20" t="inlineStr"/>
+      <c r="S9" s="20" t="inlineStr"/>
+      <c r="T9" s="20" t="inlineStr"/>
+      <c r="U9" s="20" t="inlineStr"/>
+      <c r="V9" s="20" t="inlineStr"/>
+      <c r="W9" s="20" t="inlineStr"/>
+      <c r="X9" s="20" t="inlineStr"/>
+      <c r="Y9" s="20" t="inlineStr"/>
+      <c r="Z9" s="20" t="inlineStr"/>
+      <c r="AA9" s="20" t="inlineStr"/>
+      <c r="AB9" s="20" t="inlineStr"/>
+      <c r="AC9" s="20" t="inlineStr"/>
+      <c r="AD9" s="20" t="inlineStr"/>
+      <c r="AE9" s="20" t="inlineStr"/>
+      <c r="AF9" s="20" t="inlineStr"/>
+      <c r="AG9" s="20" t="inlineStr"/>
     </row>
     <row r="10" ht="15.75" customFormat="1" customHeight="1" s="10">
       <c r="A10" s="9" t="n">
@@ -1906,41 +1890,37 @@
           <t>ตรวจสอบ Digital  read out และการทำงานของ Linear  scale</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n"/>
-      <c r="D10" s="20" t="n"/>
-      <c r="E10" s="20" t="n"/>
-      <c r="F10" s="20" t="n"/>
-      <c r="G10" s="20" t="n"/>
-      <c r="H10" s="20" t="n"/>
-      <c r="I10" s="20" t="n"/>
-      <c r="J10" s="20" t="n"/>
-      <c r="K10" s="20" t="n"/>
-      <c r="L10" s="20" t="n"/>
-      <c r="M10" s="20" t="n"/>
-      <c r="N10" s="20" t="n"/>
-      <c r="O10" s="20" t="n"/>
-      <c r="P10" s="20" t="n"/>
-      <c r="Q10" s="20" t="n"/>
-      <c r="R10" s="20" t="n"/>
-      <c r="S10" s="20" t="n"/>
-      <c r="T10" s="20" t="n"/>
-      <c r="U10" s="20" t="n"/>
-      <c r="V10" s="20" t="n"/>
-      <c r="W10" s="20" t="n"/>
-      <c r="X10" s="20" t="n"/>
-      <c r="Y10" s="20" t="n"/>
-      <c r="Z10" s="20" t="n"/>
-      <c r="AA10" s="20" t="n"/>
-      <c r="AB10" s="20" t="n"/>
-      <c r="AC10" s="20" t="n"/>
-      <c r="AD10" s="20" t="n"/>
-      <c r="AE10" s="20" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF10" s="20" t="n"/>
-      <c r="AG10" s="20" t="n"/>
+      <c r="C10" s="20" t="inlineStr"/>
+      <c r="D10" s="20" t="inlineStr"/>
+      <c r="E10" s="20" t="inlineStr"/>
+      <c r="F10" s="20" t="inlineStr"/>
+      <c r="G10" s="20" t="inlineStr"/>
+      <c r="H10" s="20" t="inlineStr"/>
+      <c r="I10" s="20" t="inlineStr"/>
+      <c r="J10" s="20" t="inlineStr"/>
+      <c r="K10" s="20" t="inlineStr"/>
+      <c r="L10" s="20" t="inlineStr"/>
+      <c r="M10" s="20" t="inlineStr"/>
+      <c r="N10" s="20" t="inlineStr"/>
+      <c r="O10" s="20" t="inlineStr"/>
+      <c r="P10" s="20" t="inlineStr"/>
+      <c r="Q10" s="20" t="inlineStr"/>
+      <c r="R10" s="20" t="inlineStr"/>
+      <c r="S10" s="20" t="inlineStr"/>
+      <c r="T10" s="20" t="inlineStr"/>
+      <c r="U10" s="20" t="inlineStr"/>
+      <c r="V10" s="20" t="inlineStr"/>
+      <c r="W10" s="20" t="inlineStr"/>
+      <c r="X10" s="20" t="inlineStr"/>
+      <c r="Y10" s="20" t="inlineStr"/>
+      <c r="Z10" s="20" t="inlineStr"/>
+      <c r="AA10" s="20" t="inlineStr"/>
+      <c r="AB10" s="20" t="inlineStr"/>
+      <c r="AC10" s="20" t="inlineStr"/>
+      <c r="AD10" s="20" t="inlineStr"/>
+      <c r="AE10" s="20" t="inlineStr"/>
+      <c r="AF10" s="20" t="inlineStr"/>
+      <c r="AG10" s="20" t="inlineStr"/>
     </row>
     <row r="11" ht="15.75" customFormat="1" customHeight="1" s="10">
       <c r="A11" s="9" t="n">
@@ -1951,41 +1931,37 @@
           <t>อัดจาระบีตามจุดที่อัดจาระบีทุกๆจุด</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n"/>
-      <c r="D11" s="20" t="n"/>
-      <c r="E11" s="20" t="n"/>
-      <c r="F11" s="20" t="n"/>
-      <c r="G11" s="20" t="n"/>
-      <c r="H11" s="20" t="n"/>
-      <c r="I11" s="20" t="n"/>
-      <c r="J11" s="20" t="n"/>
-      <c r="K11" s="20" t="n"/>
-      <c r="L11" s="20" t="n"/>
-      <c r="M11" s="20" t="n"/>
-      <c r="N11" s="20" t="n"/>
-      <c r="O11" s="20" t="n"/>
-      <c r="P11" s="20" t="n"/>
-      <c r="Q11" s="20" t="n"/>
-      <c r="R11" s="20" t="n"/>
-      <c r="S11" s="20" t="n"/>
-      <c r="T11" s="20" t="n"/>
-      <c r="U11" s="20" t="n"/>
-      <c r="V11" s="20" t="n"/>
-      <c r="W11" s="20" t="n"/>
-      <c r="X11" s="20" t="n"/>
-      <c r="Y11" s="20" t="n"/>
-      <c r="Z11" s="20" t="n"/>
-      <c r="AA11" s="20" t="n"/>
-      <c r="AB11" s="20" t="n"/>
-      <c r="AC11" s="20" t="n"/>
-      <c r="AD11" s="20" t="n"/>
-      <c r="AE11" s="20" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF11" s="20" t="n"/>
-      <c r="AG11" s="20" t="n"/>
+      <c r="C11" s="20" t="inlineStr"/>
+      <c r="D11" s="20" t="inlineStr"/>
+      <c r="E11" s="20" t="inlineStr"/>
+      <c r="F11" s="20" t="inlineStr"/>
+      <c r="G11" s="20" t="inlineStr"/>
+      <c r="H11" s="20" t="inlineStr"/>
+      <c r="I11" s="20" t="inlineStr"/>
+      <c r="J11" s="20" t="inlineStr"/>
+      <c r="K11" s="20" t="inlineStr"/>
+      <c r="L11" s="20" t="inlineStr"/>
+      <c r="M11" s="20" t="inlineStr"/>
+      <c r="N11" s="20" t="inlineStr"/>
+      <c r="O11" s="20" t="inlineStr"/>
+      <c r="P11" s="20" t="inlineStr"/>
+      <c r="Q11" s="20" t="inlineStr"/>
+      <c r="R11" s="20" t="inlineStr"/>
+      <c r="S11" s="20" t="inlineStr"/>
+      <c r="T11" s="20" t="inlineStr"/>
+      <c r="U11" s="20" t="inlineStr"/>
+      <c r="V11" s="20" t="inlineStr"/>
+      <c r="W11" s="20" t="inlineStr"/>
+      <c r="X11" s="20" t="inlineStr"/>
+      <c r="Y11" s="20" t="inlineStr"/>
+      <c r="Z11" s="20" t="inlineStr"/>
+      <c r="AA11" s="20" t="inlineStr"/>
+      <c r="AB11" s="20" t="inlineStr"/>
+      <c r="AC11" s="20" t="inlineStr"/>
+      <c r="AD11" s="20" t="inlineStr"/>
+      <c r="AE11" s="20" t="inlineStr"/>
+      <c r="AF11" s="20" t="inlineStr"/>
+      <c r="AG11" s="20" t="inlineStr"/>
     </row>
     <row r="12" ht="15.75" customFormat="1" customHeight="1" s="10">
       <c r="A12" s="9" t="n">
@@ -1996,41 +1972,37 @@
           <t>ตรวจสอบใบมีด  บนและล่าง</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n"/>
-      <c r="D12" s="20" t="n"/>
-      <c r="E12" s="20" t="n"/>
-      <c r="F12" s="20" t="n"/>
-      <c r="G12" s="20" t="n"/>
-      <c r="H12" s="20" t="n"/>
-      <c r="I12" s="20" t="n"/>
-      <c r="J12" s="20" t="n"/>
-      <c r="K12" s="20" t="n"/>
-      <c r="L12" s="20" t="n"/>
-      <c r="M12" s="20" t="n"/>
-      <c r="N12" s="20" t="n"/>
-      <c r="O12" s="20" t="n"/>
-      <c r="P12" s="20" t="n"/>
-      <c r="Q12" s="20" t="n"/>
-      <c r="R12" s="20" t="n"/>
-      <c r="S12" s="20" t="n"/>
-      <c r="T12" s="20" t="n"/>
-      <c r="U12" s="20" t="n"/>
-      <c r="V12" s="20" t="n"/>
-      <c r="W12" s="20" t="n"/>
-      <c r="X12" s="20" t="n"/>
-      <c r="Y12" s="20" t="n"/>
-      <c r="Z12" s="20" t="n"/>
-      <c r="AA12" s="20" t="n"/>
-      <c r="AB12" s="20" t="n"/>
-      <c r="AC12" s="20" t="n"/>
-      <c r="AD12" s="20" t="n"/>
-      <c r="AE12" s="20" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="AF12" s="20" t="n"/>
-      <c r="AG12" s="20" t="n"/>
+      <c r="C12" s="20" t="inlineStr"/>
+      <c r="D12" s="20" t="inlineStr"/>
+      <c r="E12" s="20" t="inlineStr"/>
+      <c r="F12" s="20" t="inlineStr"/>
+      <c r="G12" s="20" t="inlineStr"/>
+      <c r="H12" s="20" t="inlineStr"/>
+      <c r="I12" s="20" t="inlineStr"/>
+      <c r="J12" s="20" t="inlineStr"/>
+      <c r="K12" s="20" t="inlineStr"/>
+      <c r="L12" s="20" t="inlineStr"/>
+      <c r="M12" s="20" t="inlineStr"/>
+      <c r="N12" s="20" t="inlineStr"/>
+      <c r="O12" s="20" t="inlineStr"/>
+      <c r="P12" s="20" t="inlineStr"/>
+      <c r="Q12" s="20" t="inlineStr"/>
+      <c r="R12" s="20" t="inlineStr"/>
+      <c r="S12" s="20" t="inlineStr"/>
+      <c r="T12" s="20" t="inlineStr"/>
+      <c r="U12" s="20" t="inlineStr"/>
+      <c r="V12" s="20" t="inlineStr"/>
+      <c r="W12" s="20" t="inlineStr"/>
+      <c r="X12" s="20" t="inlineStr"/>
+      <c r="Y12" s="20" t="inlineStr"/>
+      <c r="Z12" s="20" t="inlineStr"/>
+      <c r="AA12" s="20" t="inlineStr"/>
+      <c r="AB12" s="20" t="inlineStr"/>
+      <c r="AC12" s="20" t="inlineStr"/>
+      <c r="AD12" s="20" t="inlineStr"/>
+      <c r="AE12" s="20" t="inlineStr"/>
+      <c r="AF12" s="20" t="inlineStr"/>
+      <c r="AG12" s="20" t="inlineStr"/>
     </row>
     <row r="13" ht="15.75" customFormat="1" customHeight="1" s="10">
       <c r="A13" s="9" t="n">
@@ -2041,76 +2013,72 @@
           <t xml:space="preserve">ตรวจสอบความพร้อมสภาพโดยรวมของเครื่อง จักรและอุปกรณ์เสริมต่าง ๆ </t>
         </is>
       </c>
-      <c r="C13" s="20" t="n"/>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="20" t="n"/>
-      <c r="F13" s="20" t="n"/>
-      <c r="G13" s="20" t="n"/>
-      <c r="H13" s="20" t="n"/>
-      <c r="I13" s="20" t="n"/>
-      <c r="J13" s="20" t="n"/>
-      <c r="K13" s="20" t="n"/>
-      <c r="L13" s="20" t="n"/>
-      <c r="M13" s="20" t="n"/>
-      <c r="N13" s="20" t="n"/>
-      <c r="O13" s="20" t="n"/>
-      <c r="P13" s="20" t="n"/>
-      <c r="Q13" s="20" t="n"/>
-      <c r="R13" s="20" t="n"/>
-      <c r="S13" s="20" t="n"/>
-      <c r="T13" s="20" t="n"/>
-      <c r="U13" s="20" t="n"/>
-      <c r="V13" s="20" t="n"/>
-      <c r="W13" s="20" t="n"/>
-      <c r="X13" s="20" t="n"/>
-      <c r="Y13" s="20" t="n"/>
-      <c r="Z13" s="20" t="n"/>
-      <c r="AA13" s="20" t="n"/>
-      <c r="AB13" s="20" t="n"/>
-      <c r="AC13" s="20" t="n"/>
-      <c r="AD13" s="20" t="n"/>
-      <c r="AE13" s="39" t="inlineStr">
-        <is>
-          <t>พรมมา คาวไธสงค์</t>
-        </is>
-      </c>
-      <c r="AF13" s="20" t="n"/>
-      <c r="AG13" s="20" t="n"/>
+      <c r="C13" s="20" t="inlineStr"/>
+      <c r="D13" s="20" t="inlineStr"/>
+      <c r="E13" s="20" t="inlineStr"/>
+      <c r="F13" s="20" t="inlineStr"/>
+      <c r="G13" s="20" t="inlineStr"/>
+      <c r="H13" s="20" t="inlineStr"/>
+      <c r="I13" s="20" t="inlineStr"/>
+      <c r="J13" s="20" t="inlineStr"/>
+      <c r="K13" s="20" t="inlineStr"/>
+      <c r="L13" s="20" t="inlineStr"/>
+      <c r="M13" s="20" t="inlineStr"/>
+      <c r="N13" s="20" t="inlineStr"/>
+      <c r="O13" s="20" t="inlineStr"/>
+      <c r="P13" s="20" t="inlineStr"/>
+      <c r="Q13" s="20" t="inlineStr"/>
+      <c r="R13" s="20" t="inlineStr"/>
+      <c r="S13" s="20" t="inlineStr"/>
+      <c r="T13" s="20" t="inlineStr"/>
+      <c r="U13" s="20" t="inlineStr"/>
+      <c r="V13" s="20" t="inlineStr"/>
+      <c r="W13" s="20" t="inlineStr"/>
+      <c r="X13" s="20" t="inlineStr"/>
+      <c r="Y13" s="20" t="inlineStr"/>
+      <c r="Z13" s="20" t="inlineStr"/>
+      <c r="AA13" s="20" t="inlineStr"/>
+      <c r="AB13" s="20" t="inlineStr"/>
+      <c r="AC13" s="20" t="inlineStr"/>
+      <c r="AD13" s="20" t="inlineStr"/>
+      <c r="AE13" s="39" t="inlineStr"/>
+      <c r="AF13" s="20" t="inlineStr"/>
+      <c r="AG13" s="20" t="inlineStr"/>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="8" t="n"/>
       <c r="B14" s="7" t="n"/>
-      <c r="C14" s="23" t="n"/>
-      <c r="D14" s="23" t="n"/>
-      <c r="E14" s="23" t="n"/>
-      <c r="F14" s="23" t="n"/>
-      <c r="G14" s="23" t="n"/>
-      <c r="H14" s="23" t="n"/>
-      <c r="I14" s="23" t="n"/>
-      <c r="J14" s="23" t="n"/>
-      <c r="K14" s="23" t="n"/>
-      <c r="L14" s="23" t="n"/>
-      <c r="M14" s="23" t="n"/>
-      <c r="N14" s="23" t="n"/>
-      <c r="O14" s="23" t="n"/>
-      <c r="P14" s="23" t="n"/>
-      <c r="Q14" s="23" t="n"/>
-      <c r="R14" s="23" t="n"/>
-      <c r="S14" s="23" t="n"/>
-      <c r="T14" s="23" t="n"/>
-      <c r="U14" s="23" t="n"/>
-      <c r="V14" s="23" t="n"/>
-      <c r="W14" s="23" t="n"/>
-      <c r="X14" s="23" t="n"/>
-      <c r="Y14" s="23" t="n"/>
-      <c r="Z14" s="23" t="n"/>
-      <c r="AA14" s="37" t="n"/>
-      <c r="AB14" s="23" t="n"/>
-      <c r="AC14" s="23" t="n"/>
-      <c r="AD14" s="23" t="n"/>
-      <c r="AE14" s="23" t="n"/>
-      <c r="AF14" s="23" t="n"/>
-      <c r="AG14" s="23" t="n"/>
+      <c r="C14" s="23" t="inlineStr"/>
+      <c r="D14" s="23" t="inlineStr"/>
+      <c r="E14" s="23" t="inlineStr"/>
+      <c r="F14" s="23" t="inlineStr"/>
+      <c r="G14" s="23" t="inlineStr"/>
+      <c r="H14" s="23" t="inlineStr"/>
+      <c r="I14" s="23" t="inlineStr"/>
+      <c r="J14" s="23" t="inlineStr"/>
+      <c r="K14" s="23" t="inlineStr"/>
+      <c r="L14" s="23" t="inlineStr"/>
+      <c r="M14" s="23" t="inlineStr"/>
+      <c r="N14" s="23" t="inlineStr"/>
+      <c r="O14" s="23" t="inlineStr"/>
+      <c r="P14" s="23" t="inlineStr"/>
+      <c r="Q14" s="23" t="inlineStr"/>
+      <c r="R14" s="23" t="inlineStr"/>
+      <c r="S14" s="23" t="inlineStr"/>
+      <c r="T14" s="23" t="inlineStr"/>
+      <c r="U14" s="23" t="inlineStr"/>
+      <c r="V14" s="23" t="inlineStr"/>
+      <c r="W14" s="23" t="inlineStr"/>
+      <c r="X14" s="23" t="inlineStr"/>
+      <c r="Y14" s="23" t="inlineStr"/>
+      <c r="Z14" s="23" t="inlineStr"/>
+      <c r="AA14" s="37" t="inlineStr"/>
+      <c r="AB14" s="23" t="inlineStr"/>
+      <c r="AC14" s="23" t="inlineStr"/>
+      <c r="AD14" s="23" t="inlineStr"/>
+      <c r="AE14" s="23" t="inlineStr"/>
+      <c r="AF14" s="23" t="inlineStr"/>
+      <c r="AG14" s="23" t="inlineStr"/>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="B15" s="6" t="n"/>
@@ -2214,7 +2182,9 @@
       <c r="AF17" s="24" t="n"/>
       <c r="AG17" s="24" t="n"/>
     </row>
-    <row r="18" ht="12" customHeight="1"/>
+    <row r="18" ht="12" customHeight="1">
+      <c r="B18" t="inlineStr"/>
+    </row>
     <row r="19" ht="19.5" customHeight="1">
       <c r="B19" s="17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Direct Write Excel for CUTTING-01 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_CUTTING-01.xlsx
+++ b/FM-MN-07_CUTTING-01.xlsx
@@ -1731,7 +1731,11 @@
       <c r="E6" s="20" t="inlineStr"/>
       <c r="F6" s="20" t="inlineStr"/>
       <c r="G6" s="20" t="inlineStr"/>
-      <c r="H6" s="20" t="inlineStr"/>
+      <c r="H6" s="20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I6" s="20" t="inlineStr"/>
       <c r="J6" s="20" t="inlineStr"/>
       <c r="K6" s="20" t="inlineStr"/>
@@ -1772,7 +1776,11 @@
       <c r="E7" s="20" t="inlineStr"/>
       <c r="F7" s="20" t="inlineStr"/>
       <c r="G7" s="20" t="inlineStr"/>
-      <c r="H7" s="20" t="inlineStr"/>
+      <c r="H7" s="20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I7" s="20" t="inlineStr"/>
       <c r="J7" s="20" t="inlineStr"/>
       <c r="K7" s="20" t="inlineStr"/>
@@ -1813,7 +1821,11 @@
       <c r="E8" s="20" t="inlineStr"/>
       <c r="F8" s="20" t="inlineStr"/>
       <c r="G8" s="20" t="inlineStr"/>
-      <c r="H8" s="20" t="inlineStr"/>
+      <c r="H8" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="20" t="inlineStr"/>
       <c r="J8" s="20" t="inlineStr"/>
       <c r="K8" s="20" t="inlineStr"/>
@@ -1854,7 +1866,11 @@
       <c r="E9" s="20" t="inlineStr"/>
       <c r="F9" s="20" t="inlineStr"/>
       <c r="G9" s="20" t="inlineStr"/>
-      <c r="H9" s="20" t="inlineStr"/>
+      <c r="H9" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="20" t="inlineStr"/>
       <c r="J9" s="20" t="inlineStr"/>
       <c r="K9" s="20" t="inlineStr"/>
@@ -1895,7 +1911,11 @@
       <c r="E10" s="20" t="inlineStr"/>
       <c r="F10" s="20" t="inlineStr"/>
       <c r="G10" s="20" t="inlineStr"/>
-      <c r="H10" s="20" t="inlineStr"/>
+      <c r="H10" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="20" t="inlineStr"/>
       <c r="J10" s="20" t="inlineStr"/>
       <c r="K10" s="20" t="inlineStr"/>
@@ -1936,7 +1956,11 @@
       <c r="E11" s="20" t="inlineStr"/>
       <c r="F11" s="20" t="inlineStr"/>
       <c r="G11" s="20" t="inlineStr"/>
-      <c r="H11" s="20" t="inlineStr"/>
+      <c r="H11" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I11" s="20" t="inlineStr"/>
       <c r="J11" s="20" t="inlineStr"/>
       <c r="K11" s="20" t="inlineStr"/>
@@ -1977,7 +2001,11 @@
       <c r="E12" s="20" t="inlineStr"/>
       <c r="F12" s="20" t="inlineStr"/>
       <c r="G12" s="20" t="inlineStr"/>
-      <c r="H12" s="20" t="inlineStr"/>
+      <c r="H12" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I12" s="20" t="inlineStr"/>
       <c r="J12" s="20" t="inlineStr"/>
       <c r="K12" s="20" t="inlineStr"/>
@@ -2018,7 +2046,11 @@
       <c r="E13" s="20" t="inlineStr"/>
       <c r="F13" s="20" t="inlineStr"/>
       <c r="G13" s="20" t="inlineStr"/>
-      <c r="H13" s="20" t="inlineStr"/>
+      <c r="H13" s="39" t="inlineStr">
+        <is>
+          <t>วชิรทย์</t>
+        </is>
+      </c>
       <c r="I13" s="20" t="inlineStr"/>
       <c r="J13" s="20" t="inlineStr"/>
       <c r="K13" s="20" t="inlineStr"/>
@@ -2182,9 +2214,7 @@
       <c r="AF17" s="24" t="n"/>
       <c r="AG17" s="24" t="n"/>
     </row>
-    <row r="18" ht="12" customHeight="1">
-      <c r="B18" t="inlineStr"/>
-    </row>
+    <row r="18" ht="12" customHeight="1"/>
     <row r="19" ht="19.5" customHeight="1">
       <c r="B19" s="17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CUTTING-01 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_CUTTING-01.xlsx
+++ b/FM-MN-07_CUTTING-01.xlsx
@@ -1736,7 +1736,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I6" s="20" t="inlineStr"/>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J6" s="20" t="inlineStr"/>
       <c r="K6" s="20" t="inlineStr"/>
       <c r="L6" s="20" t="inlineStr"/>
@@ -1781,7 +1785,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I7" s="20" t="inlineStr"/>
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J7" s="20" t="inlineStr"/>
       <c r="K7" s="20" t="inlineStr"/>
       <c r="L7" s="20" t="inlineStr"/>
@@ -1826,7 +1834,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="20" t="inlineStr"/>
+      <c r="I8" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="20" t="inlineStr"/>
       <c r="K8" s="20" t="inlineStr"/>
       <c r="L8" s="20" t="inlineStr"/>
@@ -1871,7 +1883,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="20" t="inlineStr"/>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="20" t="inlineStr"/>
       <c r="K9" s="20" t="inlineStr"/>
       <c r="L9" s="20" t="inlineStr"/>
@@ -1916,7 +1932,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="20" t="inlineStr"/>
+      <c r="I10" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="20" t="inlineStr"/>
       <c r="K10" s="20" t="inlineStr"/>
       <c r="L10" s="20" t="inlineStr"/>
@@ -1961,7 +1981,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I11" s="20" t="inlineStr"/>
+      <c r="I11" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J11" s="20" t="inlineStr"/>
       <c r="K11" s="20" t="inlineStr"/>
       <c r="L11" s="20" t="inlineStr"/>
@@ -2006,7 +2030,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I12" s="20" t="inlineStr"/>
+      <c r="I12" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J12" s="20" t="inlineStr"/>
       <c r="K12" s="20" t="inlineStr"/>
       <c r="L12" s="20" t="inlineStr"/>
@@ -2051,7 +2079,11 @@
           <t>วชิรทย์</t>
         </is>
       </c>
-      <c r="I13" s="20" t="inlineStr"/>
+      <c r="I13" s="39" t="inlineStr">
+        <is>
+          <t>วชิรวิทย์</t>
+        </is>
+      </c>
       <c r="J13" s="20" t="inlineStr"/>
       <c r="K13" s="20" t="inlineStr"/>
       <c r="L13" s="20" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CUTTING-01 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_CUTTING-01.xlsx
+++ b/FM-MN-07_CUTTING-01.xlsx
@@ -1741,7 +1741,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J6" s="20" t="inlineStr"/>
+      <c r="J6" s="20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="K6" s="20" t="inlineStr"/>
       <c r="L6" s="20" t="inlineStr"/>
       <c r="M6" s="20" t="inlineStr"/>
@@ -1790,7 +1794,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J7" s="20" t="inlineStr"/>
+      <c r="J7" s="20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="K7" s="20" t="inlineStr"/>
       <c r="L7" s="20" t="inlineStr"/>
       <c r="M7" s="20" t="inlineStr"/>
@@ -1839,7 +1847,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="20" t="inlineStr"/>
+      <c r="J8" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="20" t="inlineStr"/>
       <c r="L8" s="20" t="inlineStr"/>
       <c r="M8" s="20" t="inlineStr"/>
@@ -1888,7 +1900,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="20" t="inlineStr"/>
+      <c r="J9" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="20" t="inlineStr"/>
       <c r="L9" s="20" t="inlineStr"/>
       <c r="M9" s="20" t="inlineStr"/>
@@ -1937,7 +1953,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="20" t="inlineStr"/>
+      <c r="J10" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="20" t="inlineStr"/>
       <c r="L10" s="20" t="inlineStr"/>
       <c r="M10" s="20" t="inlineStr"/>
@@ -1986,7 +2006,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J11" s="20" t="inlineStr"/>
+      <c r="J11" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K11" s="20" t="inlineStr"/>
       <c r="L11" s="20" t="inlineStr"/>
       <c r="M11" s="20" t="inlineStr"/>
@@ -2035,7 +2059,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J12" s="20" t="inlineStr"/>
+      <c r="J12" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K12" s="20" t="inlineStr"/>
       <c r="L12" s="20" t="inlineStr"/>
       <c r="M12" s="20" t="inlineStr"/>
@@ -2084,7 +2112,11 @@
           <t>วชิรวิทย์</t>
         </is>
       </c>
-      <c r="J13" s="20" t="inlineStr"/>
+      <c r="J13" s="39" t="inlineStr">
+        <is>
+          <t>วชิรวิทย์</t>
+        </is>
+      </c>
       <c r="K13" s="20" t="inlineStr"/>
       <c r="L13" s="20" t="inlineStr"/>
       <c r="M13" s="20" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for CUTTING-01 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_CUTTING-01.xlsx
+++ b/FM-MN-07_CUTTING-01.xlsx
@@ -1747,7 +1747,11 @@
         </is>
       </c>
       <c r="K6" s="20" t="inlineStr"/>
-      <c r="L6" s="20" t="inlineStr"/>
+      <c r="L6" s="20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="M6" s="20" t="inlineStr"/>
       <c r="N6" s="20" t="inlineStr"/>
       <c r="O6" s="20" t="inlineStr"/>
@@ -1800,7 +1804,11 @@
         </is>
       </c>
       <c r="K7" s="20" t="inlineStr"/>
-      <c r="L7" s="20" t="inlineStr"/>
+      <c r="L7" s="20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="M7" s="20" t="inlineStr"/>
       <c r="N7" s="20" t="inlineStr"/>
       <c r="O7" s="20" t="inlineStr"/>
@@ -1853,7 +1861,11 @@
         </is>
       </c>
       <c r="K8" s="20" t="inlineStr"/>
-      <c r="L8" s="20" t="inlineStr"/>
+      <c r="L8" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="20" t="inlineStr"/>
       <c r="N8" s="20" t="inlineStr"/>
       <c r="O8" s="20" t="inlineStr"/>
@@ -1906,7 +1918,11 @@
         </is>
       </c>
       <c r="K9" s="20" t="inlineStr"/>
-      <c r="L9" s="20" t="inlineStr"/>
+      <c r="L9" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="20" t="inlineStr"/>
       <c r="N9" s="20" t="inlineStr"/>
       <c r="O9" s="20" t="inlineStr"/>
@@ -1959,7 +1975,11 @@
         </is>
       </c>
       <c r="K10" s="20" t="inlineStr"/>
-      <c r="L10" s="20" t="inlineStr"/>
+      <c r="L10" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="20" t="inlineStr"/>
       <c r="N10" s="20" t="inlineStr"/>
       <c r="O10" s="20" t="inlineStr"/>
@@ -2012,7 +2032,11 @@
         </is>
       </c>
       <c r="K11" s="20" t="inlineStr"/>
-      <c r="L11" s="20" t="inlineStr"/>
+      <c r="L11" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M11" s="20" t="inlineStr"/>
       <c r="N11" s="20" t="inlineStr"/>
       <c r="O11" s="20" t="inlineStr"/>
@@ -2065,7 +2089,11 @@
         </is>
       </c>
       <c r="K12" s="20" t="inlineStr"/>
-      <c r="L12" s="20" t="inlineStr"/>
+      <c r="L12" s="20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M12" s="20" t="inlineStr"/>
       <c r="N12" s="20" t="inlineStr"/>
       <c r="O12" s="20" t="inlineStr"/>
@@ -2118,7 +2146,11 @@
         </is>
       </c>
       <c r="K13" s="20" t="inlineStr"/>
-      <c r="L13" s="20" t="inlineStr"/>
+      <c r="L13" s="39" t="inlineStr">
+        <is>
+          <t>วชิรวิทย์</t>
+        </is>
+      </c>
       <c r="M13" s="20" t="inlineStr"/>
       <c r="N13" s="20" t="inlineStr"/>
       <c r="O13" s="20" t="inlineStr"/>

</xml_diff>